<commit_message>
feat: expand Zoho export coverage to 16 templates
Add Journal, Vendor Credits, Customer/Vendor Payment, Expense, Deposit,
and Bank Transfer mappers (previously out of scope for lack of a
template), and widen Invoice/Bill/Credit Note to match Zoho's newer,
much larger bulk-import column sets (GST split, billing/shipping
blocks, bill-allocation detail). Wires all 7 new entities through
full-sync mapping, single-job export, and bulk export.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/src/mapping/templates/Item.xlsx
+++ b/backend/src/mapping/templates/Item.xlsx
@@ -1,26 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Silver Tech Expert\Desktop\Tally to excel\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{6DC6177C-B763-4C4A-9401-3FCDA3503EF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420"/>
   </bookViews>
   <sheets>
-    <sheet name="Item" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Item" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="118">
   <si>
     <t>Item ID</t>
   </si>
@@ -223,6 +217,9 @@
     <t>Cost Centre</t>
   </si>
   <si>
+    <t>Stock Group</t>
+  </si>
+  <si>
     <t>Dummy Item</t>
   </si>
   <si>
@@ -289,6 +286,9 @@
     <t>INR 97.45</t>
   </si>
   <si>
+    <t>service</t>
+  </si>
+  <si>
     <t>GST12</t>
   </si>
   <si>
@@ -368,333 +368,30 @@
   </si>
   <si>
     <t>INR 0.00</t>
-  </si>
-  <si>
-    <t>service</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri Light"/>
-      <family val="2"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C5700"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="10">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -702,204 +399,15 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.39997558519241921"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="42">
-    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1211,10 +719,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BO6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:BP6"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <sheetData>
-    <row r="1" spans="1:67" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1416,19 +924,22 @@
       <c r="BO1" t="s">
         <v>66</v>
       </c>
+      <c r="BP1" t="s">
+        <v>67</v>
+      </c>
     </row>
-    <row r="2" spans="1:67" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>2.8113490000010701E+18</v>
+        <v>2811349000001070000</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C2">
         <v>1234</v>
       </c>
       <c r="D2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I2" t="b">
         <v>1</v>
@@ -1440,10 +951,10 @@
         <v>0</v>
       </c>
       <c r="O2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="P2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="R2">
         <v>0</v>
@@ -1458,67 +969,67 @@
         <v>0</v>
       </c>
       <c r="V2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="W2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Y2" t="b">
         <v>1</v>
       </c>
       <c r="AB2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="AC2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="AK2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="AL2">
         <v>18</v>
       </c>
       <c r="AM2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="AN2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="AO2">
         <v>18</v>
       </c>
       <c r="AP2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="AQ2">
         <v>1</v>
       </c>
       <c r="AT2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="AU2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="AV2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="AW2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="AX2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="BA2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="BC2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="BH2">
         <v>0</v>
       </c>
       <c r="BI2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="BJ2" t="b">
         <v>1</v>
@@ -1536,18 +1047,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:67" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>2.8113490000013599E+18</v>
+        <v>2811349000001360000</v>
       </c>
       <c r="B3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E3">
         <v>901396165224</v>
@@ -1559,7 +1070,7 @@
         <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="L3">
         <v>34022090</v>
@@ -1568,10 +1079,10 @@
         <v>0</v>
       </c>
       <c r="O3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="P3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="R3">
         <v>0</v>
@@ -1586,61 +1097,61 @@
         <v>0</v>
       </c>
       <c r="V3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="W3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Y3" t="b">
         <v>1</v>
       </c>
       <c r="AB3" t="s">
-        <v>116</v>
+        <v>90</v>
       </c>
       <c r="AC3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AK3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AL3">
         <v>12</v>
       </c>
       <c r="AM3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="AN3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="AO3">
         <v>12</v>
       </c>
       <c r="AP3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="AQ3">
         <v>1</v>
       </c>
       <c r="AT3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="AU3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="AV3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="AW3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="AX3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="BA3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="BC3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="BD3">
         <v>250</v>
@@ -1649,7 +1160,7 @@
         <v>0</v>
       </c>
       <c r="BI3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="BJ3" t="b">
         <v>1</v>
@@ -1667,12 +1178,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:67" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>2.8113490000013701E+18</v>
+        <v>2811349000001370000</v>
       </c>
       <c r="B4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -1681,19 +1192,19 @@
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="K4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="M4" t="b">
         <v>0</v>
       </c>
       <c r="O4" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="P4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="R4">
         <v>0</v>
@@ -1708,79 +1219,79 @@
         <v>0</v>
       </c>
       <c r="V4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="W4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Y4" t="b">
         <v>1</v>
       </c>
       <c r="AB4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="AC4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AE4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="AF4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="AG4" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="AH4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="AI4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="AJ4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="AK4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AL4">
         <v>12</v>
       </c>
       <c r="AM4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="AN4" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="AO4">
         <v>12</v>
       </c>
       <c r="AP4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="AQ4">
         <v>1</v>
       </c>
       <c r="AT4" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="AU4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="AV4" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="AW4" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="AX4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="BA4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="BC4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="BD4">
         <v>100</v>
@@ -1789,7 +1300,7 @@
         <v>0</v>
       </c>
       <c r="BI4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="BJ4" t="b">
         <v>1</v>
@@ -1807,15 +1318,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:67" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>2.8113490000016901E+18</v>
+        <v>2811349000001690000</v>
       </c>
       <c r="B5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="I5" t="b">
         <v>1</v>
@@ -1824,10 +1335,10 @@
         <v>0</v>
       </c>
       <c r="O5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="P5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="R5">
         <v>0</v>
@@ -1842,64 +1353,64 @@
         <v>0</v>
       </c>
       <c r="V5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="W5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Y5" t="b">
         <v>1</v>
       </c>
       <c r="AB5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="AC5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="AK5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AL5">
         <v>12</v>
       </c>
       <c r="AM5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="AN5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="AO5">
         <v>12</v>
       </c>
       <c r="AP5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="AQ5">
         <v>1</v>
       </c>
       <c r="AT5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="AU5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="AW5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="AX5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="BA5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="BC5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="BH5">
         <v>0</v>
       </c>
       <c r="BI5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="BJ5" t="b">
         <v>1</v>
@@ -1917,15 +1428,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:67" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>2.8113490000024202E+18</v>
+        <v>2811349000002420000</v>
       </c>
       <c r="B6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="I6" t="b">
         <v>0</v>
@@ -1934,10 +1445,10 @@
         <v>0</v>
       </c>
       <c r="O6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="R6">
         <v>0</v>
@@ -1952,52 +1463,52 @@
         <v>0</v>
       </c>
       <c r="V6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="W6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Y6" t="b">
         <v>1</v>
       </c>
       <c r="AB6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="AC6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="AK6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AL6">
         <v>12</v>
       </c>
       <c r="AM6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="AN6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="AO6">
         <v>12</v>
       </c>
       <c r="AP6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="AQ6">
         <v>5</v>
       </c>
       <c r="AT6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="AU6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="AW6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="BI6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="BJ6" t="b">
         <v>1</v>

</xml_diff>